<commit_message>
Publish approved listing-review investment ranges.
Operator-approved 초투 updates Golden 실투자금, the spec, and the app datasets. Held zones keep their previous ranges.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/archive/golden/zone_rollup.xlsx
+++ b/data/archive/golden/zone_rollup.xlsx
@@ -10,7 +10,7 @@
     <sheet name="구역통합본" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'구역통합본'!$A$1:$O$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'구역통합본'!$A$1:$O$60</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O56"/>
+  <dimension ref="A1:O60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -544,440 +544,440 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>동작구</t>
+          <t>금천구</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>사당동</t>
+          <t>독산동</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>사당 12구역</t>
+          <t>독산시흥구역</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>추진위 승인</t>
+          <t>조합설립인가</t>
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>1.55</v>
+        <v>2.35</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>4.1</v>
+        <v>6.58</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>2.5</v>
+        <v>2.35</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>4.1</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="J2" s="2" t="n"/>
       <c r="K2" s="2" t="n"/>
       <c r="L2" s="3" t="n">
-        <v>1.55</v>
+        <v>2.35</v>
       </c>
       <c r="M2" s="3" t="n">
-        <v>4.1</v>
+        <v>6.58</v>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>2.5~4.1</t>
+          <t>6.58~9.3</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>동작구|사당동|사당 12구역</t>
+          <t>금천구|독산동|독산시흥구역</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>동작구</t>
+          <t>금천구</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>상도동</t>
+          <t>독산동</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>상도 21구역(모아타운)</t>
+          <t>독산 2구역</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>(모아)관리계획고시</t>
+          <t>조합설립인가</t>
         </is>
       </c>
       <c r="E3" s="2" t="n">
         <v>5</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>1.8</v>
+        <v>2.73</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>3.9</v>
+        <v>7.97</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>1.8</v>
+        <v>4.3</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>3.9</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="J3" s="2" t="n"/>
       <c r="K3" s="2" t="n"/>
       <c r="L3" s="3" t="n">
-        <v>1.8</v>
+        <v>2.73</v>
       </c>
       <c r="M3" s="3" t="n">
-        <v>3.9</v>
+        <v>8.15</v>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>1.8~3.9</t>
+          <t>4.8~10.7</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>동작구|상도동|상도 21구역(모아타운)</t>
+          <t>금천구|독산동|독산 2구역</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>중랑구</t>
+          <t>구리시</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>중화동</t>
+          <t>수택동</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>중화 6구역</t>
+          <t>수택 2구역</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>정비구역지정</t>
+          <t>시공사 선정</t>
         </is>
       </c>
       <c r="E4" s="2" t="n">
         <v>5</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>9.699999999999999</v>
+        <v>3.7</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>3.5</v>
+        <v>4.2</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="J4" s="2" t="n"/>
       <c r="K4" s="2" t="n"/>
       <c r="L4" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M4" s="3" t="n">
-        <v>9.699999999999999</v>
+        <v>5</v>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>3.5~10</t>
+          <t>3.1~3.9</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>중랑구|중화동|중화 6구역</t>
+          <t>구리시|수택동|수택 2구역</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>구리시</t>
+          <t>성북구</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>수택동</t>
+          <t>장위동</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>수택 2구역</t>
+          <t>장위 13-2구역</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>조합설립인가</t>
+          <t>정비구역지정</t>
         </is>
       </c>
       <c r="E5" s="2" t="n">
         <v>5</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>2.4</v>
+        <v>3.28</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>2.9</v>
+        <v>4</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>3.1</v>
+        <v>4.4</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>3.9</v>
+        <v>4.6</v>
       </c>
       <c r="J5" s="2" t="n"/>
       <c r="K5" s="2" t="n"/>
       <c r="L5" s="3" t="n">
-        <v>2.4</v>
+        <v>1.8</v>
       </c>
       <c r="M5" s="3" t="n">
-        <v>2.9</v>
+        <v>2</v>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>3.1~3.9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>구리시|수택동|수택 2구역</t>
+          <t>성북구|장위동|장위 13-2구역</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>금천구</t>
+          <t>광진구</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>독산동</t>
+          <t>자양동</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>독산시흥구역</t>
+          <t>자양1동 799(모아타운)</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>조합설립인가</t>
+          <t>(모아)관리계획고시</t>
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>3.35</v>
+        <v>3.5</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>9.300000000000001</v>
+        <v>5.7</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>6.58</v>
+        <v>3.5</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>9.300000000000001</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="J6" s="2" t="n"/>
       <c r="K6" s="2" t="n"/>
       <c r="L6" s="3" t="n">
-        <v>3.35</v>
+        <v>3.5</v>
       </c>
       <c r="M6" s="3" t="n">
-        <v>9.300000000000001</v>
+        <v>7.5</v>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>6.58~9.3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>금천구|독산동|독산시흥구역</t>
+          <t>광진구|자양동|자양1동 799(모아타운)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>용산구</t>
+          <t>강북구</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>청파동</t>
+          <t>미아동</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>청파 2구역</t>
+          <t>미아 2구역</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>조합설립인가</t>
+          <t>건축심의</t>
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>3.8</v>
+        <v>4.2</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>8.1</v>
+        <v>6.48</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>4.5</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>8.1</v>
+        <v>6.65</v>
       </c>
       <c r="J7" s="2" t="n"/>
       <c r="K7" s="2" t="n"/>
       <c r="L7" s="3" t="n">
-        <v>3.8</v>
+        <v>4.2</v>
       </c>
       <c r="M7" s="3" t="n">
-        <v>8.1</v>
+        <v>6.48</v>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>4.5~8.1</t>
+          <t>7.5~12.5</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>용산구|청파동|청파 2구역</t>
+          <t>강북구|미아동|미아 2구역</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>동작구</t>
+          <t>중랑구</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>상도동</t>
+          <t>중화동</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>상도 16구역</t>
+          <t>중화 6구역</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>추진위 승인</t>
+          <t>정비구역지정</t>
         </is>
       </c>
       <c r="E8" s="2" t="n">
         <v>5</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>3.9</v>
+        <v>4.6</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>3.9</v>
+        <v>4.6</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="J8" s="2" t="n"/>
       <c r="K8" s="2" t="n"/>
       <c r="L8" s="3" t="n">
-        <v>3.9</v>
+        <v>4.6</v>
       </c>
       <c r="M8" s="3" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>3.9~4</t>
+          <t>3.5~10</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>동작구|상도동|상도 16구역</t>
+          <t>중랑구|중화동|중화 6구역</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>금천구</t>
+          <t>강북구</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>독산동</t>
+          <t>미아동</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>독산 2구역</t>
+          <t>미아 9-2구역(재건축)</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>조합설립인가</t>
+          <t>사업시행인가</t>
         </is>
       </c>
       <c r="E9" s="2" t="n">
         <v>5</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>4.8</v>
+        <v>5.5</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>8.800000000000001</v>
+        <v>7.5</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>4.8</v>
+        <v>6</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>10.7</v>
+        <v>8</v>
       </c>
       <c r="J9" s="2" t="n"/>
       <c r="K9" s="2" t="n"/>
       <c r="L9" s="3" t="n">
-        <v>4.8</v>
+        <v>5.4</v>
       </c>
       <c r="M9" s="3" t="n">
-        <v>8.800000000000001</v>
+        <v>10</v>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>4.8~10.7</t>
+          <t>6~10</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>금천구|독산동|독산 2구역</t>
+          <t>강북구|미아동|미아 9-2구역(재건축)</t>
         </is>
       </c>
     </row>
@@ -989,54 +989,54 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>길음동</t>
+          <t>장위동</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>길음 5구역</t>
+          <t>장위 14구역</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>조합설립인가</t>
+          <t>시공사 선정</t>
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>5.2</v>
+        <v>5.5</v>
       </c>
       <c r="G10" s="3" t="n">
         <v>6</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>6</v>
+        <v>5.5</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>7.3</v>
+        <v>7.1</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>1.33</v>
+        <v>1</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>1.33</v>
+        <v>1</v>
       </c>
       <c r="L10" s="3" t="n">
-        <v>5.2</v>
+        <v>5.5</v>
       </c>
       <c r="M10" s="3" t="n">
-        <v>6</v>
+        <v>6.2</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>6~7.3</t>
+          <t>5.5~6.2</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>성북구|길음동|길음 5구역</t>
+          <t>성북구|장위동|장위 14구역</t>
         </is>
       </c>
     </row>
@@ -1048,160 +1048,160 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>장위동</t>
+          <t>길음동</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>장위 15구역</t>
+          <t>길음 5구역</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>시공사 선정</t>
+          <t>조합설립인가</t>
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>5.25</v>
+        <v>5.8</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>7.1</v>
+        <v>6</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>7</v>
+        <v>5.8</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J11" s="2" t="n"/>
       <c r="K11" s="2" t="n"/>
       <c r="L11" s="3" t="n">
-        <v>5.25</v>
+        <v>5.8</v>
       </c>
       <c r="M11" s="3" t="n">
-        <v>7.1</v>
+        <v>6.3</v>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>7~8</t>
+          <t>6~7.3</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>성북구|장위동|장위 15구역</t>
+          <t>성북구|길음동|길음 5구역</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>강북구</t>
+          <t>동작구</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>미아동</t>
+          <t>상도동</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>미아 9-2구역(재건축)</t>
+          <t>상도 15구역</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>사업시행인가</t>
+          <t>시공사 선정</t>
         </is>
       </c>
       <c r="E12" s="2" t="n">
         <v>5</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>5.4</v>
+        <v>5.86</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>10</v>
+        <v>7.15</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>6</v>
+        <v>6.5</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>10</v>
+        <v>7.5</v>
       </c>
       <c r="J12" s="2" t="n"/>
       <c r="K12" s="2" t="n"/>
       <c r="L12" s="3" t="n">
-        <v>5.4</v>
+        <v>5.86</v>
       </c>
       <c r="M12" s="3" t="n">
-        <v>10</v>
+        <v>7.3</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>6~10</t>
+          <t>8~9.6</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>강북구|미아동|미아 9-2구역(재건축)</t>
+          <t>동작구|상도동|상도 15구역</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>성북구</t>
+          <t>금천구</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>장위동</t>
+          <t>독산동</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>장위 14구역</t>
+          <t>독산 1구역</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>시공사 선정</t>
+          <t>사업시행자 지정</t>
         </is>
       </c>
       <c r="E13" s="2" t="n">
         <v>5</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>5.5</v>
+        <v>5.9</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>5.98</v>
+        <v>11.2</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>5.5</v>
+        <v>7.2</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>6.2</v>
+        <v>13</v>
       </c>
       <c r="J13" s="2" t="n"/>
       <c r="K13" s="2" t="n"/>
       <c r="L13" s="3" t="n">
-        <v>5.5</v>
+        <v>5.9</v>
       </c>
       <c r="M13" s="3" t="n">
-        <v>5.98</v>
+        <v>11.8</v>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>5.5~6.2</t>
+          <t>6.9~12</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>성북구|장위동|장위 14구역</t>
+          <t>금천구|독산동|독산 1구역</t>
         </is>
       </c>
     </row>
@@ -1218,71 +1218,71 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>신흥 3구역</t>
+          <t>신흥 1구역</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>시공사 선정</t>
+          <t>사업시행인가</t>
         </is>
       </c>
       <c r="E14" s="2" t="n">
         <v>5</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>5.6</v>
+        <v>5.9</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>7.3</v>
+        <v>8.5</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>7.5</v>
+        <v>8</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>8.6</v>
+        <v>9.5</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>4.05</v>
+        <v>4</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>4.7</v>
+        <v>5.18</v>
       </c>
       <c r="L14" s="3" t="n">
-        <v>5.6</v>
+        <v>5.9</v>
       </c>
       <c r="M14" s="3" t="n">
-        <v>7.3</v>
+        <v>8.5</v>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>7.5~8.6</t>
+          <t>7.3~8.3</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>성남시 수정구|신흥동|신흥 3구역</t>
+          <t>성남시 수정구|신흥동|신흥 1구역</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>용산구</t>
+          <t>성남시 수정구</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>청파동</t>
+          <t>수진동</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>서계통합</t>
+          <t>수진 1구역</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>조합설립인가</t>
+          <t>관리처분인가</t>
         </is>
       </c>
       <c r="E15" s="2" t="n">
@@ -1292,47 +1292,51 @@
         <v>6</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>9.800000000000001</v>
+        <v>8.6</v>
       </c>
       <c r="H15" s="3" t="n">
-        <v>7</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="I15" s="3" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="J15" s="2" t="n"/>
-      <c r="K15" s="2" t="n"/>
+        <v>10.22</v>
+      </c>
+      <c r="J15" s="3" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="K15" s="3" t="n">
+        <v>5.68</v>
+      </c>
       <c r="L15" s="3" t="n">
         <v>6</v>
       </c>
       <c r="M15" s="3" t="n">
-        <v>9.800000000000001</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>7~9.8</t>
+          <t>8.29~9.5</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>용산구|청파동|서계통합</t>
+          <t>성남시 수정구|수진동|수진 1구역</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>강북구</t>
+          <t>용산구</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>미아동</t>
+          <t>청파동</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>미아 2구역</t>
+          <t>서계통합</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -1344,481 +1348,477 @@
         <v>5</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>6.2</v>
+        <v>6</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>10.5</v>
+        <v>12</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>7.5</v>
+        <v>7</v>
       </c>
       <c r="I16" s="3" t="n">
-        <v>12.5</v>
-      </c>
-      <c r="J16" s="2" t="n"/>
-      <c r="K16" s="2" t="n"/>
+        <v>12</v>
+      </c>
+      <c r="J16" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="K16" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="L16" s="3" t="n">
-        <v>6.2</v>
+        <v>6</v>
       </c>
       <c r="M16" s="3" t="n">
-        <v>10.5</v>
+        <v>12</v>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>7.5~12.5</t>
+          <t>7~9.8</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>강북구|미아동|미아 2구역</t>
+          <t>용산구|청파동|서계통합</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>은평구</t>
+          <t>성북구</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>갈현동</t>
+          <t>장위동</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>갈현 1구역</t>
+          <t>장위 15구역</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>관리처분인가</t>
+          <t>시공사 선정</t>
         </is>
       </c>
       <c r="E17" s="2" t="n">
         <v>5</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>6.8</v>
+        <v>6.25</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>7.06</v>
+        <v>7.5</v>
       </c>
       <c r="H17" s="3" t="n">
-        <v>6.8</v>
+        <v>6.9</v>
       </c>
       <c r="I17" s="3" t="n">
-        <v>7.06</v>
+        <v>9</v>
       </c>
       <c r="J17" s="2" t="n"/>
       <c r="K17" s="2" t="n"/>
       <c r="L17" s="3" t="n">
-        <v>6.8</v>
+        <v>6.25</v>
       </c>
       <c r="M17" s="3" t="n">
-        <v>7.06</v>
+        <v>7.5</v>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>6.8~7.06</t>
+          <t>7~8</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>은평구|갈현동|갈현 1구역</t>
+          <t>성북구|장위동|장위 15구역</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>동작구</t>
+          <t>성북구</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>상도동</t>
+          <t>길음동</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>상도 14구역</t>
+          <t>신길음구역</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>사업시행자 지정</t>
+          <t>사업시행인가</t>
         </is>
       </c>
       <c r="E18" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>6.8</v>
+        <v>6.3</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>8.6</v>
+        <v>6.3</v>
       </c>
       <c r="H18" s="3" t="n">
-        <v>7.5</v>
+        <v>6.5</v>
       </c>
       <c r="I18" s="3" t="n">
-        <v>8.6</v>
+        <v>6.5</v>
       </c>
       <c r="J18" s="2" t="n"/>
       <c r="K18" s="2" t="n"/>
       <c r="L18" s="3" t="n">
-        <v>6.8</v>
+        <v>6.3</v>
       </c>
       <c r="M18" s="3" t="n">
-        <v>8.6</v>
+        <v>6.3</v>
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>7.5~8.6</t>
+          <t>8.5</t>
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>동작구|상도동|상도 14구역</t>
+          <t>성북구|길음동|신길음구역</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>금천구</t>
+          <t>성남시 수정구</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>독산동</t>
+          <t>신흥동</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>독산 1구역</t>
+          <t>신흥 3구역</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>사업시행자 지정</t>
+          <t>시공사 선정</t>
         </is>
       </c>
       <c r="E19" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>6.9</v>
+        <v>7</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>11.8</v>
+        <v>8.6</v>
       </c>
       <c r="H19" s="3" t="n">
-        <v>6.9</v>
+        <v>8.6</v>
       </c>
       <c r="I19" s="3" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="J19" s="2" t="n"/>
       <c r="K19" s="2" t="n"/>
       <c r="L19" s="3" t="n">
-        <v>6.9</v>
+        <v>7.3</v>
       </c>
       <c r="M19" s="3" t="n">
-        <v>11.8</v>
+        <v>8.6</v>
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>6.9~12</t>
+          <t>7.5~8.6</t>
         </is>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>금천구|독산동|독산 1구역</t>
+          <t>성남시 수정구|신흥동|신흥 3구역</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>광진구</t>
+          <t>은평구</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>자양동</t>
+          <t>갈현동</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>자양2동 649(B)(모아타운)</t>
+          <t>갈현 1구역</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>(모아)관리계획고시</t>
+          <t>관리처분인가</t>
         </is>
       </c>
       <c r="E20" s="2" t="n">
         <v>5</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>6.9</v>
+        <v>7.08</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>7.8</v>
+        <v>7.1</v>
       </c>
       <c r="H20" s="3" t="n">
-        <v>9</v>
+        <v>7.08</v>
       </c>
       <c r="I20" s="3" t="n">
-        <v>9</v>
+        <v>7.1</v>
       </c>
       <c r="J20" s="2" t="n"/>
       <c r="K20" s="2" t="n"/>
       <c r="L20" s="3" t="n">
-        <v>6.9</v>
+        <v>7.08</v>
       </c>
       <c r="M20" s="3" t="n">
-        <v>7.8</v>
+        <v>7.1</v>
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6.8~7.06</t>
         </is>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>광진구|자양동|자양2동 649(B)(모아타운)</t>
+          <t>은평구|갈현동|갈현 1구역</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>성남시 수정구</t>
+          <t>동작구</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>수진동</t>
+          <t>상도동</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>수진 1구역</t>
+          <t>상도 14구역</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>관리처분인가</t>
+          <t>사업시행자 지정</t>
         </is>
       </c>
       <c r="E21" s="2" t="n">
         <v>5</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>6.9</v>
+        <v>7.5</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>7.58</v>
+        <v>9.5</v>
       </c>
       <c r="H21" s="3" t="n">
-        <v>8.289999999999999</v>
+        <v>7.5</v>
       </c>
       <c r="I21" s="3" t="n">
         <v>9.5</v>
       </c>
-      <c r="J21" s="3" t="n">
-        <v>4.68</v>
-      </c>
-      <c r="K21" s="3" t="n">
-        <v>4.68</v>
-      </c>
+      <c r="J21" s="2" t="n"/>
+      <c r="K21" s="2" t="n"/>
       <c r="L21" s="3" t="n">
-        <v>6.9</v>
+        <v>7.5</v>
       </c>
       <c r="M21" s="3" t="n">
-        <v>7.58</v>
+        <v>9.5</v>
       </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t>8.29~9.5</t>
+          <t>7.5~8.6</t>
         </is>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>성남시 수정구|수진동|수진 1구역</t>
+          <t>동작구|상도동|상도 14구역</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>성남시 수정구</t>
+          <t>용산구</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>신흥동</t>
+          <t>청파동</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>신흥 1구역</t>
+          <t>청파 1구역</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>사업시행인가</t>
+          <t>조합설립인가</t>
         </is>
       </c>
       <c r="E22" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>7</v>
+        <v>7.5</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>7.6</v>
+        <v>16.5</v>
       </c>
       <c r="H22" s="3" t="n">
-        <v>7.3</v>
+        <v>7.5</v>
       </c>
       <c r="I22" s="3" t="n">
-        <v>8.300000000000001</v>
-      </c>
-      <c r="J22" s="3" t="n">
-        <v>4.6</v>
-      </c>
-      <c r="K22" s="3" t="n">
-        <v>4.6</v>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="J22" s="2" t="n"/>
+      <c r="K22" s="2" t="n"/>
       <c r="L22" s="3" t="n">
-        <v>7</v>
+        <v>7.5</v>
       </c>
       <c r="M22" s="3" t="n">
-        <v>7.6</v>
+        <v>16.5</v>
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>7.3~8.3</t>
+          <t>7.5~20</t>
         </is>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>성남시 수정구|신흥동|신흥 1구역</t>
+          <t>용산구|청파동|청파 1구역</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>동작구</t>
+          <t>마포구</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>사당동</t>
+          <t>공덕동</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>사당 5구역(재건축)</t>
+          <t>공덕 8구역</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>사업시행인가</t>
+          <t>추진위 승인</t>
         </is>
       </c>
       <c r="E23" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>7.5</v>
+        <v>7.62</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>12</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="H23" s="3" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="I23" s="3" t="n">
         <v>10</v>
-      </c>
-      <c r="I23" s="3" t="n">
-        <v>12</v>
       </c>
       <c r="J23" s="2" t="n"/>
       <c r="K23" s="2" t="n"/>
       <c r="L23" s="3" t="n">
-        <v>7.5</v>
+        <v>7.62</v>
       </c>
       <c r="M23" s="3" t="n">
-        <v>12</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t>10~12</t>
+          <t>8.5</t>
         </is>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>동작구|사당동|사당 5구역(재건축)</t>
+          <t>마포구|공덕동|공덕 8구역</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>용산구</t>
+          <t>영등포구</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>청파동</t>
+          <t>신길동</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>청파 1구역</t>
+          <t>신길 16-2구역</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>조합설립인가</t>
+          <t>정비구역지정</t>
         </is>
       </c>
       <c r="E24" s="2" t="n">
         <v>5</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>7.5</v>
+        <v>7.7</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="H24" s="3" t="n">
-        <v>7.5</v>
+        <v>9.1</v>
       </c>
       <c r="I24" s="3" t="n">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="J24" s="2" t="n"/>
       <c r="K24" s="2" t="n"/>
       <c r="L24" s="3" t="n">
-        <v>7.5</v>
+        <v>7.7</v>
       </c>
       <c r="M24" s="3" t="n">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>7.5~20</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>용산구|청파동|청파 1구역</t>
+          <t>영등포구|신길동|신길 16-2구역</t>
         </is>
       </c>
     </row>
@@ -1830,147 +1830,143 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>공덕동</t>
+          <t>염리동</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>공덕 8구역</t>
+          <t>염리 5구역</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>추진위 승인</t>
+          <t>정비구역지정</t>
         </is>
       </c>
       <c r="E25" s="2" t="n">
         <v>5</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>7.62</v>
+        <v>7.8</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>8.199999999999999</v>
+        <v>7.8</v>
       </c>
       <c r="H25" s="3" t="n">
-        <v>8.5</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="I25" s="3" t="n">
-        <v>8.5</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="J25" s="2" t="n"/>
       <c r="K25" s="2" t="n"/>
       <c r="L25" s="3" t="n">
-        <v>7.62</v>
+        <v>7.8</v>
       </c>
       <c r="M25" s="3" t="n">
-        <v>8.199999999999999</v>
+        <v>9.9</v>
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>8.5</t>
+          <t>9.3~12</t>
         </is>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>마포구|공덕동|공덕 8구역</t>
+          <t>마포구|염리동|염리 5구역</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>마포구</t>
+          <t>광진구</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>염리동</t>
+          <t>자양동</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>염리 5구역</t>
+          <t>자양동 772-1(건대모아)</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>정비구역지정</t>
+          <t>조합설립인가</t>
         </is>
       </c>
       <c r="E26" s="2" t="n">
         <v>5</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>7.8</v>
+        <v>8</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>24.85</v>
+        <v>13</v>
       </c>
       <c r="H26" s="3" t="n">
-        <v>9.300000000000001</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="I26" s="3" t="n">
-        <v>37</v>
-      </c>
-      <c r="J26" s="3" t="n">
-        <v>12.7</v>
-      </c>
-      <c r="K26" s="3" t="n">
-        <v>12.7</v>
-      </c>
+        <v>13</v>
+      </c>
+      <c r="J26" s="2" t="n"/>
+      <c r="K26" s="2" t="n"/>
       <c r="L26" s="3" t="n">
-        <v>7.8</v>
+        <v>8</v>
       </c>
       <c r="M26" s="3" t="n">
-        <v>24.85</v>
+        <v>13</v>
       </c>
       <c r="N26" s="2" t="inlineStr">
         <is>
-          <t>9.3~37</t>
+          <t>6.7~7.5</t>
         </is>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>마포구|염리동|염리 5구역</t>
+          <t>광진구|자양동|자양동 772-1(건대모아)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>동작구</t>
+          <t>동대문구</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>상도동</t>
+          <t>제기동</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>상도 15구역</t>
+          <t>제기 6구역</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>시공사 선정</t>
+          <t>관리처분인가</t>
         </is>
       </c>
       <c r="E27" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F27" s="3" t="n">
         <v>8</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>9.6</v>
+        <v>8</v>
       </c>
       <c r="H27" s="3" t="n">
-        <v>8</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="I27" s="3" t="n">
-        <v>9.6</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="J27" s="2" t="n"/>
       <c r="K27" s="2" t="n"/>
@@ -1978,51 +1974,51 @@
         <v>8</v>
       </c>
       <c r="M27" s="3" t="n">
-        <v>9.6</v>
+        <v>8</v>
       </c>
       <c r="N27" s="2" t="inlineStr">
         <is>
-          <t>8~9.6</t>
+          <t>9.8</t>
         </is>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>동작구|상도동|상도 15구역</t>
+          <t>동대문구|제기동|제기 6구역</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>성북구</t>
+          <t>용산구</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>길음동</t>
+          <t>청파동</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>신길음구역</t>
+          <t>청파 2구역</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>사업시행인가</t>
+          <t>조합설립인가</t>
         </is>
       </c>
       <c r="E28" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>8.5</v>
+        <v>8</v>
       </c>
       <c r="G28" s="3" t="n">
         <v>8.5</v>
       </c>
       <c r="H28" s="3" t="n">
-        <v>8.5</v>
+        <v>8</v>
       </c>
       <c r="I28" s="3" t="n">
         <v>8.5</v>
@@ -2030,260 +2026,264 @@
       <c r="J28" s="2" t="n"/>
       <c r="K28" s="2" t="n"/>
       <c r="L28" s="3" t="n">
-        <v>8.5</v>
+        <v>8</v>
       </c>
       <c r="M28" s="3" t="n">
         <v>8.5</v>
       </c>
       <c r="N28" s="2" t="inlineStr">
         <is>
-          <t>8.5</t>
+          <t>8~8.1</t>
         </is>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>성북구|길음동|신길음구역</t>
+          <t>용산구|청파동|청파 2구역</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>영등포구</t>
+          <t>용산구</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>신길동</t>
+          <t>이촌동</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>신길 2구역</t>
+          <t>이촌1구역(재건축)</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>사업시행인가</t>
+          <t>정비구역지정</t>
         </is>
       </c>
       <c r="E29" s="2" t="n">
         <v>5</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>8.5</v>
+        <v>8.390000000000001</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>13.87</v>
+        <v>14</v>
       </c>
       <c r="H29" s="3" t="n">
-        <v>8.5</v>
+        <v>9</v>
       </c>
       <c r="I29" s="3" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="J29" s="2" t="n"/>
+      <c r="K29" s="2" t="n"/>
+      <c r="L29" s="3" t="n">
+        <v>8.390000000000001</v>
+      </c>
+      <c r="M29" s="3" t="n">
         <v>14</v>
       </c>
-      <c r="J29" s="3" t="n">
-        <v>3.8</v>
-      </c>
-      <c r="K29" s="3" t="n">
-        <v>3.8</v>
-      </c>
-      <c r="L29" s="3" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="M29" s="3" t="n">
-        <v>13.87</v>
-      </c>
       <c r="N29" s="2" t="inlineStr">
         <is>
-          <t>8.5~14</t>
+          <t>12~14.2</t>
         </is>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>영등포구|신길동|신길 2구역</t>
+          <t>용산구|이촌동|이촌1구역(재건축)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>광진구</t>
+          <t>마포구</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>자양동</t>
+          <t>공덕동</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>자양동 227-147</t>
+          <t>공덕 7구역</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>정비구역지정</t>
+          <t>조합설립인가</t>
         </is>
       </c>
       <c r="E30" s="2" t="n">
         <v>5</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>9</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>10.25</v>
+        <v>12.8</v>
       </c>
       <c r="H30" s="3" t="n">
-        <v>10.5</v>
+        <v>10</v>
       </c>
       <c r="I30" s="3" t="n">
-        <v>12.5</v>
-      </c>
-      <c r="J30" s="2" t="n"/>
-      <c r="K30" s="2" t="n"/>
+        <v>14</v>
+      </c>
+      <c r="J30" s="3" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="K30" s="3" t="n">
+        <v>6.4</v>
+      </c>
       <c r="L30" s="3" t="n">
-        <v>9</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="M30" s="3" t="n">
-        <v>10.25</v>
+        <v>13.8</v>
       </c>
       <c r="N30" s="2" t="inlineStr">
         <is>
-          <t>10.5~12.5</t>
+          <t>11~13</t>
         </is>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>광진구|자양동|자양동 227-147</t>
+          <t>마포구|공덕동|공덕 7구역</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>은평구</t>
+          <t>광진구</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>불광동</t>
+          <t>자양동</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>불광 5구역</t>
+          <t>자양2동 649(B)(모아타운)</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>관리처분인가</t>
+          <t>조합설립인가</t>
         </is>
       </c>
       <c r="E31" s="2" t="n">
         <v>5</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>9.17</v>
+        <v>9</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>10.52</v>
+        <v>12</v>
       </c>
       <c r="H31" s="3" t="n">
-        <v>9.17</v>
+        <v>9.6</v>
       </c>
       <c r="I31" s="3" t="n">
-        <v>10.52</v>
-      </c>
-      <c r="J31" s="2" t="n"/>
-      <c r="K31" s="2" t="n"/>
+        <v>13</v>
+      </c>
+      <c r="J31" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="K31" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="L31" s="3" t="n">
-        <v>9.17</v>
+        <v>6.9</v>
       </c>
       <c r="M31" s="3" t="n">
-        <v>10.52</v>
+        <v>7.8</v>
       </c>
       <c r="N31" s="2" t="inlineStr">
         <is>
-          <t>9.17~10.52</t>
+          <t>9</t>
         </is>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
-          <t>은평구|불광동|불광 5구역</t>
+          <t>광진구|자양동|자양2동 649(B)(모아타운)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>송파구</t>
+          <t>은평구</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>마천동</t>
+          <t>불광동</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>마천 1구역</t>
+          <t>불광 5구역</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>조합설립인가</t>
+          <t>관리처분인가</t>
         </is>
       </c>
       <c r="E32" s="2" t="n">
         <v>5</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>9.199999999999999</v>
+        <v>9.17</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>11</v>
+        <v>10.52</v>
       </c>
       <c r="H32" s="3" t="n">
-        <v>11</v>
+        <v>9.17</v>
       </c>
       <c r="I32" s="3" t="n">
-        <v>13</v>
+        <v>10.52</v>
       </c>
       <c r="J32" s="2" t="n"/>
       <c r="K32" s="2" t="n"/>
       <c r="L32" s="3" t="n">
-        <v>9.199999999999999</v>
+        <v>9.17</v>
       </c>
       <c r="M32" s="3" t="n">
-        <v>11</v>
+        <v>10.52</v>
       </c>
       <c r="N32" s="2" t="inlineStr">
         <is>
-          <t>11~13</t>
+          <t>9.17~10.52</t>
         </is>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>송파구|마천동|마천 1구역</t>
+          <t>은평구|불광동|불광 5구역</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>마포구</t>
+          <t>송파구</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>공덕동</t>
+          <t>마천동</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>공덕 7구역</t>
+          <t>마천 1구역</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -2292,31 +2292,27 @@
         </is>
       </c>
       <c r="E33" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>9.48</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>11.5</v>
+        <v>10.6</v>
       </c>
       <c r="H33" s="3" t="n">
-        <v>11</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="I33" s="3" t="n">
-        <v>13</v>
-      </c>
-      <c r="J33" s="3" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="K33" s="3" t="n">
-        <v>7.4</v>
-      </c>
+        <v>11.8</v>
+      </c>
+      <c r="J33" s="2" t="n"/>
+      <c r="K33" s="2" t="n"/>
       <c r="L33" s="3" t="n">
-        <v>9.48</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="M33" s="3" t="n">
-        <v>11.5</v>
+        <v>10.6</v>
       </c>
       <c r="N33" s="2" t="inlineStr">
         <is>
@@ -2325,62 +2321,66 @@
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
-          <t>마포구|공덕동|공덕 7구역</t>
+          <t>송파구|마천동|마천 1구역</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>동대문구</t>
+          <t>송파구</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>전농동</t>
+          <t>마천동</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>전농 8구역</t>
+          <t>마천 3구역</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>조합설립인가</t>
+          <t>사업시행인가</t>
         </is>
       </c>
       <c r="E34" s="2" t="n">
         <v>5</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>9.5</v>
+        <v>9.4</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>12.55</v>
+        <v>9.51</v>
       </c>
       <c r="H34" s="3" t="n">
-        <v>11.5</v>
+        <v>10</v>
       </c>
       <c r="I34" s="3" t="n">
-        <v>12.55</v>
-      </c>
-      <c r="J34" s="2" t="n"/>
-      <c r="K34" s="2" t="n"/>
+        <v>11</v>
+      </c>
+      <c r="J34" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="K34" s="3" t="n">
+        <v>6.89</v>
+      </c>
       <c r="L34" s="3" t="n">
-        <v>9.5</v>
+        <v>9.4</v>
       </c>
       <c r="M34" s="3" t="n">
-        <v>12.55</v>
+        <v>10</v>
       </c>
       <c r="N34" s="2" t="inlineStr">
         <is>
-          <t>11.5~12.55</t>
+          <t>11~13.2</t>
         </is>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
-          <t>동대문구|전농동|전농 8구역</t>
+          <t>송파구|마천동|마천 3구역</t>
         </is>
       </c>
     </row>
@@ -2392,181 +2392,177 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>제기동</t>
+          <t>전농동</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>제기 6구역</t>
+          <t>전농 8구역</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>관리처분인가</t>
+          <t>조합설립인가</t>
         </is>
       </c>
       <c r="E35" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>9.800000000000001</v>
+        <v>9.5</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>9.800000000000001</v>
+        <v>12</v>
       </c>
       <c r="H35" s="3" t="n">
-        <v>9.800000000000001</v>
+        <v>11.5</v>
       </c>
       <c r="I35" s="3" t="n">
-        <v>9.800000000000001</v>
+        <v>12</v>
       </c>
       <c r="J35" s="2" t="n"/>
       <c r="K35" s="2" t="n"/>
       <c r="L35" s="3" t="n">
-        <v>9.800000000000001</v>
+        <v>9.5</v>
       </c>
       <c r="M35" s="3" t="n">
-        <v>9.800000000000001</v>
+        <v>12</v>
       </c>
       <c r="N35" s="2" t="inlineStr">
         <is>
-          <t>9.8</t>
+          <t>11.5~12.55</t>
         </is>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
-          <t>동대문구|제기동|제기 6구역</t>
+          <t>동대문구|전농동|전농 8구역</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>동작구</t>
+          <t>광진구</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>사당동</t>
+          <t>자양동</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>사당 17구역</t>
+          <t>자양동 227-147</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>조합설립인가</t>
+          <t>정비구역지정</t>
         </is>
       </c>
       <c r="E36" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>10</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>13.5</v>
+        <v>12</v>
       </c>
       <c r="H36" s="3" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="I36" s="3" t="n">
-        <v>13.5</v>
+        <v>13</v>
       </c>
       <c r="J36" s="2" t="n"/>
       <c r="K36" s="2" t="n"/>
       <c r="L36" s="3" t="n">
-        <v>10</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="M36" s="3" t="n">
-        <v>13.5</v>
+        <v>12</v>
       </c>
       <c r="N36" s="2" t="inlineStr">
         <is>
-          <t>10~13.5</t>
+          <t>10.5~12.5</t>
         </is>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
-          <t>동작구|사당동|사당 17구역</t>
+          <t>광진구|자양동|자양동 227-147</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>서대문구</t>
+          <t>동작구</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>북아현동</t>
+          <t>사당동</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>북아현 3구역</t>
+          <t>사당 17구역</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>사업시행인가</t>
+          <t>조합설립인가</t>
         </is>
       </c>
       <c r="E37" s="2" t="n">
         <v>5</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>10.5</v>
+        <v>10</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>13.61</v>
+        <v>18</v>
       </c>
       <c r="H37" s="3" t="n">
-        <v>10.5</v>
+        <v>10</v>
       </c>
       <c r="I37" s="3" t="n">
-        <v>23.6</v>
-      </c>
-      <c r="J37" s="3" t="n">
-        <v>10.6</v>
-      </c>
-      <c r="K37" s="3" t="n">
-        <v>12</v>
-      </c>
+        <v>18</v>
+      </c>
+      <c r="J37" s="2" t="n"/>
+      <c r="K37" s="2" t="n"/>
       <c r="L37" s="3" t="n">
-        <v>10.5</v>
+        <v>10</v>
       </c>
       <c r="M37" s="3" t="n">
-        <v>13.61</v>
+        <v>18</v>
       </c>
       <c r="N37" s="2" t="inlineStr">
         <is>
-          <t>10.5~23.6</t>
+          <t>10~13.5</t>
         </is>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
-          <t>서대문구|북아현동|북아현 3구역</t>
+          <t>동작구|사당동|사당 17구역</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>송파구</t>
+          <t>동작구</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>마천동</t>
+          <t>사당동</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>마천 3구역</t>
+          <t>사당 5구역(재건축)</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -2575,36 +2571,36 @@
         </is>
       </c>
       <c r="E38" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>10.6</v>
+        <v>10.44</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>11.5</v>
+        <v>10.44</v>
       </c>
       <c r="H38" s="3" t="n">
         <v>11</v>
       </c>
       <c r="I38" s="3" t="n">
-        <v>13.2</v>
+        <v>11</v>
       </c>
       <c r="J38" s="2" t="n"/>
       <c r="K38" s="2" t="n"/>
       <c r="L38" s="3" t="n">
-        <v>10.6</v>
+        <v>10.44</v>
       </c>
       <c r="M38" s="3" t="n">
-        <v>11.5</v>
+        <v>10.44</v>
       </c>
       <c r="N38" s="2" t="inlineStr">
         <is>
-          <t>11~13.2</t>
+          <t>10~12</t>
         </is>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
-          <t>송파구|마천동|마천 3구역</t>
+          <t>동작구|사당동|사당 5구역(재건축)</t>
         </is>
       </c>
     </row>
@@ -2626,23 +2622,23 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>추진위 승인</t>
+          <t>조합설립인가</t>
         </is>
       </c>
       <c r="E39" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F39" s="3" t="n">
         <v>10.65</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>23.5</v>
+        <v>12.3</v>
       </c>
       <c r="H39" s="3" t="n">
-        <v>13.5</v>
+        <v>13</v>
       </c>
       <c r="I39" s="3" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="J39" s="2" t="n"/>
       <c r="K39" s="2" t="n"/>
@@ -2650,11 +2646,11 @@
         <v>10.65</v>
       </c>
       <c r="M39" s="3" t="n">
-        <v>23.5</v>
+        <v>12.6</v>
       </c>
       <c r="N39" s="2" t="inlineStr">
         <is>
-          <t>13.5~24</t>
+          <t>13.5~16</t>
         </is>
       </c>
       <c r="O39" s="2" t="inlineStr">
@@ -2666,186 +2662,182 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>강북구</t>
+          <t>서대문구</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>미아동</t>
+          <t>북아현동</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>미아 4구역</t>
+          <t>북아현 3구역</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>관리처분인가</t>
+          <t>사업시행인가</t>
         </is>
       </c>
       <c r="E40" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>11.2</v>
+        <v>11.47</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>16</v>
+        <v>11.9</v>
       </c>
       <c r="H40" s="3" t="n">
-        <v>11.2</v>
+        <v>11.9</v>
       </c>
       <c r="I40" s="3" t="n">
-        <v>16</v>
-      </c>
-      <c r="J40" s="3" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="K40" s="3" t="n">
-        <v>4.5</v>
-      </c>
+        <v>13.5</v>
+      </c>
+      <c r="J40" s="2" t="n"/>
+      <c r="K40" s="2" t="n"/>
       <c r="L40" s="3" t="n">
-        <v>11.2</v>
+        <v>11.4</v>
       </c>
       <c r="M40" s="3" t="n">
-        <v>16</v>
+        <v>11.9</v>
       </c>
       <c r="N40" s="2" t="inlineStr">
         <is>
-          <t>11.2~16</t>
+          <t>13~23.6</t>
         </is>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
-          <t>강북구|미아동|미아 4구역</t>
+          <t>서대문구|북아현동|북아현 3구역</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>성동구</t>
+          <t>강북구</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>금호동3가</t>
+          <t>미아동</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>금호 21구역</t>
+          <t>미아 4구역</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>시공사 선정</t>
+          <t>관리처분인가</t>
         </is>
       </c>
       <c r="E41" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F41" s="3" t="n">
-        <v>11.8</v>
+        <v>11.5</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>16.4</v>
+        <v>12.5</v>
       </c>
       <c r="H41" s="3" t="n">
-        <v>13</v>
+        <v>11.5</v>
       </c>
       <c r="I41" s="3" t="n">
-        <v>18</v>
+        <v>12.5</v>
       </c>
       <c r="J41" s="2" t="n"/>
       <c r="K41" s="2" t="n"/>
       <c r="L41" s="3" t="n">
-        <v>11.8</v>
+        <v>11.5</v>
       </c>
       <c r="M41" s="3" t="n">
-        <v>16.4</v>
+        <v>12.5</v>
       </c>
       <c r="N41" s="2" t="inlineStr">
         <is>
-          <t>13~18</t>
+          <t>11.2~16</t>
         </is>
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
-          <t>성동구|금호동3가|금호 21구역</t>
+          <t>강북구|미아동|미아 4구역</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>강북구</t>
+          <t>성동구</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>미아동</t>
+          <t>금호동3가</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>미아 3구역</t>
+          <t>금호 21구역</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>관리처분인가</t>
+          <t>시공사 선정</t>
         </is>
       </c>
       <c r="E42" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F42" s="3" t="n">
-        <v>12</v>
+        <v>11.5</v>
       </c>
       <c r="G42" s="3" t="n">
-        <v>12</v>
+        <v>16.35</v>
       </c>
       <c r="H42" s="3" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="I42" s="3" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="J42" s="2" t="n"/>
       <c r="K42" s="2" t="n"/>
       <c r="L42" s="3" t="n">
-        <v>12</v>
+        <v>11.5</v>
       </c>
       <c r="M42" s="3" t="n">
-        <v>12</v>
+        <v>16.4</v>
       </c>
       <c r="N42" s="2" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13~18</t>
         </is>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
-          <t>강북구|미아동|미아 3구역</t>
+          <t>성동구|금호동3가|금호 21구역</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>동대문구</t>
+          <t>강북구</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>청량리동</t>
+          <t>미아동</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>청량리 8구역</t>
+          <t>미아 3구역</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -2854,7 +2846,7 @@
         </is>
       </c>
       <c r="E43" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F43" s="3" t="n">
         <v>12</v>
@@ -2868,12 +2860,8 @@
       <c r="I43" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="J43" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="K43" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="J43" s="2" t="n"/>
+      <c r="K43" s="2" t="n"/>
       <c r="L43" s="3" t="n">
         <v>12</v>
       </c>
@@ -2887,100 +2875,104 @@
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
-          <t>동대문구|청량리동|청량리 8구역</t>
+          <t>강북구|미아동|미아 3구역</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>용산구</t>
+          <t>동대문구</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>이촌동</t>
+          <t>청량리동</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>이촌1구역(재건축)</t>
+          <t>청량리 6구역</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>정비구역지정</t>
+          <t>사업시행인가</t>
         </is>
       </c>
       <c r="E44" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F44" s="3" t="n">
         <v>12</v>
       </c>
       <c r="G44" s="3" t="n">
-        <v>14.2</v>
+        <v>13.5</v>
       </c>
       <c r="H44" s="3" t="n">
         <v>12</v>
       </c>
       <c r="I44" s="3" t="n">
-        <v>14.2</v>
-      </c>
-      <c r="J44" s="2" t="n"/>
-      <c r="K44" s="2" t="n"/>
+        <v>13.5</v>
+      </c>
+      <c r="J44" s="3" t="n">
+        <v>8.15</v>
+      </c>
+      <c r="K44" s="3" t="n">
+        <v>8.15</v>
+      </c>
       <c r="L44" s="3" t="n">
         <v>12</v>
       </c>
       <c r="M44" s="3" t="n">
-        <v>14.2</v>
+        <v>13.5</v>
       </c>
       <c r="N44" s="2" t="inlineStr">
         <is>
-          <t>12~14.2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
-          <t>용산구|이촌동|이촌1구역(재건축)</t>
+          <t>동대문구|청량리동|청량리 6구역</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>중구</t>
+          <t>동대문구</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>신당동</t>
+          <t>청량리동</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>신당 10구역</t>
+          <t>청량리 8구역</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>시공사 선정</t>
+          <t>관리처분인가</t>
         </is>
       </c>
       <c r="E45" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F45" s="3" t="n">
         <v>12</v>
       </c>
       <c r="G45" s="3" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="H45" s="3" t="n">
         <v>12</v>
       </c>
       <c r="I45" s="3" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="J45" s="2" t="n"/>
       <c r="K45" s="2" t="n"/>
@@ -2988,16 +2980,16 @@
         <v>12</v>
       </c>
       <c r="M45" s="3" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="N45" s="2" t="inlineStr">
         <is>
-          <t>12~19</t>
+          <t>12</t>
         </is>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
-          <t>중구|신당동|신당 10구역</t>
+          <t>동대문구|청량리동|청량리 8구역</t>
         </is>
       </c>
     </row>
@@ -3026,24 +3018,24 @@
         <v>5</v>
       </c>
       <c r="F46" s="3" t="n">
-        <v>13</v>
+        <v>13.2</v>
       </c>
       <c r="G46" s="3" t="n">
-        <v>14.5</v>
+        <v>14.4</v>
       </c>
       <c r="H46" s="3" t="n">
-        <v>13</v>
+        <v>13.2</v>
       </c>
       <c r="I46" s="3" t="n">
-        <v>14.5</v>
+        <v>14.4</v>
       </c>
       <c r="J46" s="2" t="n"/>
       <c r="K46" s="2" t="n"/>
       <c r="L46" s="3" t="n">
-        <v>13</v>
+        <v>13.2</v>
       </c>
       <c r="M46" s="3" t="n">
-        <v>14.5</v>
+        <v>14.4</v>
       </c>
       <c r="N46" s="2" t="inlineStr">
         <is>
@@ -3059,127 +3051,127 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>용산구</t>
+          <t>성동구</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>후암동</t>
+          <t>금호동2가</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>후암1구역(재건축)</t>
+          <t>금호 16구역</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>추진위 승인</t>
+          <t>관리처분인가</t>
         </is>
       </c>
       <c r="E47" s="2" t="n">
         <v>5</v>
       </c>
       <c r="F47" s="3" t="n">
-        <v>14.5</v>
+        <v>13.26</v>
       </c>
       <c r="G47" s="3" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="H47" s="3" t="n">
-        <v>14.6</v>
+        <v>13.5</v>
       </c>
       <c r="I47" s="3" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="J47" s="2" t="n"/>
       <c r="K47" s="2" t="n"/>
       <c r="L47" s="3" t="n">
-        <v>14.5</v>
+        <v>13.26</v>
       </c>
       <c r="M47" s="3" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="N47" s="2" t="inlineStr">
         <is>
-          <t>14.6~16</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
-          <t>용산구|후암동|후암1구역(재건축)</t>
+          <t>성동구|금호동2가|금호 16구역</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>광진구</t>
+          <t>중구</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>자양동</t>
+          <t>신당동</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>자양4동 A구역</t>
+          <t>신당 10구역</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>정비구역 지정</t>
+          <t>시공사 선정</t>
         </is>
       </c>
       <c r="E48" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F48" s="3" t="n">
-        <v>15.8</v>
+        <v>14.65</v>
       </c>
       <c r="G48" s="3" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H48" s="3" t="n">
-        <v>17.5</v>
+        <v>15</v>
       </c>
       <c r="I48" s="3" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="J48" s="2" t="n"/>
       <c r="K48" s="2" t="n"/>
       <c r="L48" s="3" t="n">
-        <v>15.8</v>
+        <v>14.65</v>
       </c>
       <c r="M48" s="3" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="N48" s="2" t="inlineStr">
         <is>
-          <t>17.5~18</t>
+          <t>12~19</t>
         </is>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
-          <t>광진구|자양동|자양4동 A구역</t>
+          <t>중구|신당동|신당 10구역</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>은평구</t>
+          <t>서대문구</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>대조동</t>
+          <t>북아현동</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>대조 1구역</t>
+          <t>북아현 2구역</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
@@ -3188,36 +3180,36 @@
         </is>
       </c>
       <c r="E49" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F49" s="3" t="n">
-        <v>15.85</v>
+        <v>15.5</v>
       </c>
       <c r="G49" s="3" t="n">
-        <v>16.5</v>
+        <v>17.6</v>
       </c>
       <c r="H49" s="3" t="n">
-        <v>15.85</v>
+        <v>15.5</v>
       </c>
       <c r="I49" s="3" t="n">
-        <v>16.5</v>
+        <v>17.8</v>
       </c>
       <c r="J49" s="2" t="n"/>
       <c r="K49" s="2" t="n"/>
       <c r="L49" s="3" t="n">
-        <v>15.85</v>
+        <v>15.5</v>
       </c>
       <c r="M49" s="3" t="n">
-        <v>16.5</v>
+        <v>17.6</v>
       </c>
       <c r="N49" s="2" t="inlineStr">
         <is>
-          <t>15.85~16.5</t>
+          <t>16.86~19</t>
         </is>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
-          <t>은평구|대조동|대조 1구역</t>
+          <t>서대문구|북아현동|북아현 2구역</t>
         </is>
       </c>
     </row>
@@ -3234,104 +3226,100 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>자양 7구역</t>
+          <t>자양4동 A구역</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>조합설립인가</t>
+          <t>정비구역 지정</t>
         </is>
       </c>
       <c r="E50" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F50" s="3" t="n">
-        <v>16.1</v>
+        <v>16.4</v>
       </c>
       <c r="G50" s="3" t="n">
-        <v>17.9</v>
+        <v>18.5</v>
       </c>
       <c r="H50" s="3" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I50" s="3" t="n">
-        <v>20</v>
+        <v>18.5</v>
       </c>
       <c r="J50" s="2" t="n"/>
       <c r="K50" s="2" t="n"/>
       <c r="L50" s="3" t="n">
-        <v>16.1</v>
+        <v>16.4</v>
       </c>
       <c r="M50" s="3" t="n">
-        <v>17.9</v>
+        <v>19</v>
       </c>
       <c r="N50" s="2" t="inlineStr">
         <is>
-          <t>17~20</t>
+          <t>17.5~18</t>
         </is>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
-          <t>광진구|자양동|자양 7구역</t>
+          <t>광진구|자양동|자양4동 A구역</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>서대문구</t>
+          <t>광진구</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>북아현동</t>
+          <t>자양동</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>북아현 2구역</t>
+          <t>자양 7구역</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>관리처분인가</t>
+          <t>조합설립인가</t>
         </is>
       </c>
       <c r="E51" s="2" t="n">
         <v>5</v>
       </c>
       <c r="F51" s="3" t="n">
-        <v>16.86</v>
+        <v>17.8</v>
       </c>
       <c r="G51" s="3" t="n">
         <v>19</v>
       </c>
       <c r="H51" s="3" t="n">
-        <v>16.86</v>
+        <v>18</v>
       </c>
       <c r="I51" s="3" t="n">
-        <v>19</v>
-      </c>
-      <c r="J51" s="3" t="n">
-        <v>15</v>
-      </c>
-      <c r="K51" s="3" t="n">
-        <v>15</v>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="J51" s="2" t="n"/>
+      <c r="K51" s="2" t="n"/>
       <c r="L51" s="3" t="n">
-        <v>16.86</v>
+        <v>17.8</v>
       </c>
       <c r="M51" s="3" t="n">
         <v>19</v>
       </c>
       <c r="N51" s="2" t="inlineStr">
         <is>
-          <t>16.86~19</t>
+          <t>17~20</t>
         </is>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
-          <t>서대문구|북아현동|북아현 2구역</t>
+          <t>광진구|자양동|자양 7구역</t>
         </is>
       </c>
     </row>
@@ -3348,7 +3336,7 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>노량진 3구역</t>
+          <t>노량진 1구역</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
@@ -3357,36 +3345,36 @@
         </is>
       </c>
       <c r="E52" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F52" s="3" t="n">
-        <v>20</v>
+        <v>19.5</v>
       </c>
       <c r="G52" s="3" t="n">
-        <v>33</v>
+        <v>19.5</v>
       </c>
       <c r="H52" s="3" t="n">
-        <v>20</v>
+        <v>19.5</v>
       </c>
       <c r="I52" s="3" t="n">
-        <v>33</v>
+        <v>19.5</v>
       </c>
       <c r="J52" s="2" t="n"/>
       <c r="K52" s="2" t="n"/>
       <c r="L52" s="3" t="n">
-        <v>20</v>
+        <v>19.5</v>
       </c>
       <c r="M52" s="3" t="n">
-        <v>33</v>
+        <v>19.5</v>
       </c>
       <c r="N52" s="2" t="inlineStr">
         <is>
-          <t>20~33</t>
+          <t>20.2~27</t>
         </is>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
-          <t>동작구|노량진동|노량진 3구역</t>
+          <t>동작구|노량진동|노량진 1구역</t>
         </is>
       </c>
     </row>
@@ -3398,12 +3386,12 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>노량진동</t>
+          <t>대방동</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>노량진 1구역</t>
+          <t>노량진 7구역</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
@@ -3412,36 +3400,36 @@
         </is>
       </c>
       <c r="E53" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F53" s="3" t="n">
-        <v>20.2</v>
+        <v>19.73</v>
       </c>
       <c r="G53" s="3" t="n">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="H53" s="3" t="n">
-        <v>20.2</v>
+        <v>20</v>
       </c>
       <c r="I53" s="3" t="n">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="J53" s="2" t="n"/>
       <c r="K53" s="2" t="n"/>
       <c r="L53" s="3" t="n">
-        <v>20.2</v>
+        <v>19.73</v>
       </c>
       <c r="M53" s="3" t="n">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="N53" s="2" t="inlineStr">
         <is>
-          <t>20.2~27</t>
+          <t>21~31</t>
         </is>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
-          <t>동작구|노량진동|노량진 1구역</t>
+          <t>동작구|대방동|노량진 7구역</t>
         </is>
       </c>
     </row>
@@ -3467,27 +3455,27 @@
         </is>
       </c>
       <c r="E54" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F54" s="3" t="n">
-        <v>20.7</v>
+        <v>19.9</v>
       </c>
       <c r="G54" s="3" t="n">
-        <v>23</v>
+        <v>20.5</v>
       </c>
       <c r="H54" s="3" t="n">
-        <v>20.7</v>
+        <v>19.9</v>
       </c>
       <c r="I54" s="3" t="n">
-        <v>23</v>
+        <v>20.5</v>
       </c>
       <c r="J54" s="2" t="n"/>
       <c r="K54" s="2" t="n"/>
       <c r="L54" s="3" t="n">
-        <v>20.7</v>
+        <v>19.9</v>
       </c>
       <c r="M54" s="3" t="n">
-        <v>23</v>
+        <v>20.5</v>
       </c>
       <c r="N54" s="2" t="inlineStr">
         <is>
@@ -3508,12 +3496,12 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>대방동</t>
+          <t>노량진동</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>노량진 7구역</t>
+          <t>노량진 3구역</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
@@ -3522,100 +3510,316 @@
         </is>
       </c>
       <c r="E55" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F55" s="3" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G55" s="3" t="n">
-        <v>31</v>
+        <v>22.5</v>
       </c>
       <c r="H55" s="3" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="I55" s="3" t="n">
-        <v>31</v>
-      </c>
-      <c r="J55" s="3" t="n">
-        <v>18.1</v>
-      </c>
-      <c r="K55" s="3" t="n">
-        <v>18.1</v>
-      </c>
+        <v>27</v>
+      </c>
+      <c r="J55" s="2" t="n"/>
+      <c r="K55" s="2" t="n"/>
       <c r="L55" s="3" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M55" s="3" t="n">
-        <v>31</v>
+        <v>22.5</v>
       </c>
       <c r="N55" s="2" t="inlineStr">
         <is>
-          <t>21~31</t>
+          <t>20~33</t>
         </is>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
-          <t>동작구|대방동|노량진 7구역</t>
+          <t>동작구|노량진동|노량진 3구역</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>서초구</t>
+          <t>성동구</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>방배동</t>
+          <t>성수동</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>방배 15구역(재건축)</t>
+          <t>성수전략1구역</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>건축심의</t>
+          <t>시공사 선정</t>
         </is>
       </c>
       <c r="E56" s="2" t="n">
         <v>5</v>
       </c>
       <c r="F56" s="3" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="G56" s="3" t="n">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="H56" s="3" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="I56" s="3" t="n">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="J56" s="2" t="n"/>
       <c r="K56" s="2" t="n"/>
       <c r="L56" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="M56" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="N56" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O56" s="2" t="inlineStr">
+        <is>
+          <t>성동구|성수동|성수전략1구역</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>성동구</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>성수동</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>성수전략2구역</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>조합설립인가</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F57" s="3" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="G57" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="H57" s="3" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="I57" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="J57" s="2" t="n"/>
+      <c r="K57" s="2" t="n"/>
+      <c r="L57" s="3" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="M57" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="N57" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O57" s="2" t="inlineStr">
+        <is>
+          <t>성동구|성수동|성수전략2구역</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>성동구</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>성수동</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>성수전략3구역</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>시공사 선정</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F58" s="3" t="n">
+        <v>24.7</v>
+      </c>
+      <c r="G58" s="3" t="n">
+        <v>27.55</v>
+      </c>
+      <c r="H58" s="3" t="n">
         <v>25</v>
       </c>
-      <c r="M56" s="3" t="n">
-        <v>34</v>
-      </c>
-      <c r="N56" s="2" t="inlineStr">
+      <c r="I58" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="J58" s="2" t="n"/>
+      <c r="K58" s="2" t="n"/>
+      <c r="L58" s="3" t="n">
+        <v>24.7</v>
+      </c>
+      <c r="M58" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="N58" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O58" s="2" t="inlineStr">
+        <is>
+          <t>성동구|성수동|성수전략3구역</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>서초구</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>방배동</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>방배 15구역(재건축)</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>건축심의</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F59" s="3" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="G59" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="H59" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="I59" s="3" t="n">
+        <v>37</v>
+      </c>
+      <c r="J59" s="2" t="n"/>
+      <c r="K59" s="2" t="n"/>
+      <c r="L59" s="3" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="M59" s="3" t="n">
+        <v>33.5</v>
+      </c>
+      <c r="N59" s="2" t="inlineStr">
         <is>
           <t>25~36</t>
         </is>
       </c>
-      <c r="O56" s="2" t="inlineStr">
+      <c r="O59" s="2" t="inlineStr">
         <is>
           <t>서초구|방배동|방배 15구역(재건축)</t>
         </is>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>성동구</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>성수동</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>성수전략4구역</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>시공사 선정</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F60" s="3" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="G60" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="H60" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="I60" s="3" t="n">
+        <v>39</v>
+      </c>
+      <c r="J60" s="2" t="n"/>
+      <c r="K60" s="2" t="n"/>
+      <c r="L60" s="3" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="M60" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="N60" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O60" s="2" t="inlineStr">
+        <is>
+          <t>성동구|성수동|성수전략4구역</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O56"/>
+  <autoFilter ref="A1:O60"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>